<commit_message>
Group creation and public group list
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta Juha.xlsx
+++ b/docs/Työajan seuranta Juha.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juhaj\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5259D7C6-95DD-4E5F-BF85-67C6D89DCC80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1863FF0C-C6B9-46DE-A46E-DC392FF36B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2370" yWindow="1335" windowWidth="21600" windowHeight="11835" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11835" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Juha Jermalainen" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Ryhmä:</t>
   </si>
@@ -168,13 +168,29 @@
     <t>24.9.</t>
   </si>
   <si>
+    <t>Palaverit 
+(koko ajalta)</t>
+  </si>
+  <si>
     <t>Leffan tietosivun suunnittelu ja ensimmäinen versio
 Rajapintojen kartoitus ja linkitysten järjestely
-PR#93 tarkastus</t>
-  </si>
-  <si>
-    <t>Palaverit 
-(koko ajalta)</t>
+PR#93 tarkastus
+pr#95 tarkastus</t>
+  </si>
+  <si>
+    <t>Leffan tietosivun kommentoidut korjaukset
+Profiili sivun kommentoidut korjaukset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviews sivujen teko 
+PR#97 tarkastus
+</t>
+  </si>
+  <si>
+    <t>PR#98 tarkastus</t>
+  </si>
+  <si>
+    <t>Group sivuston teko</t>
   </si>
 </sst>
 </file>
@@ -210,19 +226,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -230,6 +240,9 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -574,228 +587,266 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="3">
         <v>1</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3</v>
+      </c>
+      <c r="E4" s="4"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="3">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="3">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="3">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="6">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="C17" s="3">
         <v>12</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="5">
-        <v>3</v>
-      </c>
-      <c r="E4" s="6"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    </row>
+    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="6">
+        <v>46291</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="6">
+        <v>46292</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="105" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="5">
-        <v>9.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="6">
+        <v>46293</v>
+      </c>
+      <c r="B20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="6">
+        <v>46294</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="3">
         <v>7</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="5">
-        <v>9.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="90" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="5">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="5">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="6"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C19" s="6"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C20" s="6"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C21" s="6"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C22" s="6"/>
+      <c r="A22" s="6"/>
+      <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C23" s="6"/>
+      <c r="A23" s="6"/>
+      <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C24" s="6"/>
+      <c r="A24" s="6"/>
+      <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C25" s="6"/>
+      <c r="A25" s="6"/>
+      <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C26" s="6"/>
+      <c r="A26" s="6"/>
+      <c r="C26" s="3"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C27" s="6"/>
+      <c r="A27" s="6"/>
+      <c r="C27" s="3"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C28" s="6"/>
+      <c r="A28" s="6"/>
+      <c r="C28" s="3"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="6"/>
+      <c r="A29" s="6"/>
+      <c r="C29" s="4"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C30" s="6"/>
+      <c r="C30" s="4"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C31" s="6"/>
+      <c r="C31" s="4"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C32" s="6"/>
+      <c r="C32" s="4"/>
     </row>
     <row r="35" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C35" s="6">
+      <c r="C35" s="4">
         <f>SUM(C3:C34,E4,E3)</f>
-        <v>78.5</v>
+        <v>93.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>